<commit_message>
cuneros y corazones actualizar
</commit_message>
<xml_diff>
--- a/data/web-repositorio.xlsx
+++ b/data/web-repositorio.xlsx
@@ -1798,7 +1798,7 @@
         <v>100</v>
       </c>
       <c r="C18" s="34">
-        <v>8000</v>
+        <v>8500</v>
       </c>
       <c r="D18" s="34">
         <v>90</v>
@@ -1827,7 +1827,7 @@
         <v>100</v>
       </c>
       <c r="C19" s="34">
-        <v>8000</v>
+        <v>8500</v>
       </c>
       <c r="D19" s="34">
         <v>90</v>
@@ -1856,7 +1856,7 @@
         <v>100</v>
       </c>
       <c r="C20" s="34">
-        <v>8000</v>
+        <v>8500</v>
       </c>
       <c r="D20" s="34">
         <v>90</v>
@@ -1886,7 +1886,7 @@
         <v>100</v>
       </c>
       <c r="C21" s="34">
-        <v>8000</v>
+        <v>8500</v>
       </c>
       <c r="D21" s="34">
         <v>50</v>

</xml_diff>